<commit_message>
fix: apply default font color to existing templates
</commit_message>
<xml_diff>
--- a/xlsx/tests/docs/COS.xlsx
+++ b/xlsx/tests/docs/COS.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\steve\Documents\IronCalc work\IronCalc-clone\IronCalc-SF\xlsx\tests\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dg-ac/Documents/IronCalc/xlsx/tests/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3FC3D82-D317-4CC6-AF82-E3B1F00A456B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AE1827E-881B-8F48-9771-407CCF049C10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14385" yWindow="-15" windowWidth="14430" windowHeight="15480" xr2:uid="{485CA009-6F4A-460D-891C-D7B8869F48AE}"/>
+    <workbookView xWindow="2280" yWindow="740" windowWidth="26540" windowHeight="15480" xr2:uid="{485CA009-6F4A-460D-891C-D7B8869F48AE}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="COS" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -67,10 +67,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="8" formatCode="&quot;£&quot;#,##0.00;[Red]\-&quot;£&quot;#,##0.00"/>
-    <numFmt numFmtId="164" formatCode="[$€-2]\ #,##0.00;\-[$€-2]\ #,##0.00"/>
+    <numFmt numFmtId="164" formatCode="&quot;£&quot;#,##0.00;[Red]\-&quot;£&quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="[$€-2]\ #,##0.00;\-[$€-2]\ #,##0.00"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -86,13 +86,32 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -107,18 +126,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -453,150 +482,156 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{698A441E-9203-46F3-91E3-D681B30E39C3}">
-  <dimension ref="A1:F12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="5" width="13.7109375" customWidth="1"/>
-    <col min="6" max="6" width="13.7109375" style="2" customWidth="1"/>
+    <col min="1" max="2" width="15.33203125" customWidth="1"/>
+    <col min="3" max="3" width="36.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.6640625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="C1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="3"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="D1" s="3"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="4">
         <f>-PI()/2</f>
         <v>-1.5707963267948966</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="4">
         <f>COS(A2)</f>
-        <v>6.1257422745431001E-17</v>
-      </c>
-      <c r="D2" t="str">
+        <v>6.123233995736766E-17</v>
+      </c>
+      <c r="C2" s="6" t="str">
         <f ca="1">_xlfn.FORMULATEXT($B2)</f>
         <v>=COS(A2)</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="4">
         <v>-0.5</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="4">
         <f>COS(A3)</f>
         <v>0.87758256189037276</v>
       </c>
-      <c r="D3" t="str">
-        <f t="shared" ref="D3:D7" ca="1" si="0">_xlfn.FORMULATEXT($B3)</f>
+      <c r="C3" s="6" t="str">
+        <f t="shared" ref="C3:C7" ca="1" si="0">_xlfn.FORMULATEXT($B3)</f>
         <v>=COS(A3)</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="4">
         <v>0</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="4">
         <f>COS(A4)</f>
         <v>1</v>
       </c>
-      <c r="D4" t="str">
+      <c r="C4" s="6" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>=COS(A4)</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="4">
         <v>0.5</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="4">
         <f>COS(A5)</f>
         <v>0.87758256189037276</v>
       </c>
-      <c r="D5" t="str">
+      <c r="C5" s="6" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>=COS(A5)</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="4">
         <f>PI()/2</f>
         <v>1.5707963267948966</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="4">
         <f>COS(A6)</f>
-        <v>6.1257422745431001E-17</v>
-      </c>
-      <c r="D6" t="str">
+        <v>6.123233995736766E-17</v>
+      </c>
+      <c r="C6" s="6" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>=COS(A6)</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B7">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="4"/>
+      <c r="B7" s="4">
         <f>COS(10*PI()/180)</f>
         <v>0.98480775301220802</v>
       </c>
-      <c r="D7" t="str">
+      <c r="C7" s="6" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>=COS(10*PI()/180)</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="4"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="6"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C9" s="1"/>
-      <c r="D9" s="1" t="s">
+      <c r="C9" s="8" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" t="e">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" s="4" t="e">
         <f>COS(SQRT(-1))</f>
         <v>#NUM!</v>
       </c>
-      <c r="B10" s="4" t="str">
+      <c r="B10" s="5" t="str">
         <f ca="1">_xlfn.FORMULATEXT($A10)</f>
         <v>=COS(SQRT(-1))</v>
       </c>
-      <c r="D10" t="s">
+      <c r="C10" s="6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" t="e">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" s="4" t="e">
         <f>COS("str")</f>
         <v>#VALUE!</v>
       </c>
-      <c r="B11" s="4" t="str">
+      <c r="B11" s="5" t="str">
         <f t="shared" ref="B11:B12" ca="1" si="1">_xlfn.FORMULATEXT($A11)</f>
         <v>=COS("str")</v>
       </c>
-      <c r="D11" t="s">
+      <c r="C11" s="6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" t="e">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" s="4" t="e">
         <f>COS(10/0)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="B12" s="4" t="str">
+      <c r="B12" s="5" t="str">
         <f t="shared" ca="1" si="1"/>
         <v>=COS(10/0)</v>
       </c>
-      <c r="D12" t="s">
+      <c r="C12" s="6" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>